<commit_message>
Create shap value importance scores
</commit_message>
<xml_diff>
--- a/Tables_Figures/average_performance_table_long.xlsx
+++ b/Tables_Figures/average_performance_table_long.xlsx
@@ -656,7 +656,7 @@
         <v>0.704481366530673</v>
       </c>
       <c r="E14" t="n">
-        <v>0.0499703900248975</v>
+        <v>0.0499703900248976</v>
       </c>
       <c r="F14" t="n">
         <v>0.032884643145528</v>
@@ -719,7 +719,7 @@
         <v>0.0998588922771032</v>
       </c>
       <c r="F17" t="n">
-        <v>0.0543728701908433</v>
+        <v>0.0543728701908434</v>
       </c>
     </row>
   </sheetData>

</xml_diff>